<commit_message>
Update project modules and test data
</commit_message>
<xml_diff>
--- a/SeleniumProject/TestData/CartData.xlsx
+++ b/SeleniumProject/TestData/CartData.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PTTKPM\THI\Gbao\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\source\repos\SeleniumProject\SeleniumProject\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C73CAD21-5ED6-47C1-99C2-6DDC4FBFD89A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07928C43-4209-48B0-9877-8FD3319FC999}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{B8ECCEAD-E6B2-46C2-B297-8A99F3AE59DD}"/>
+    <workbookView xWindow="5760" yWindow="3720" windowWidth="17280" windowHeight="9960" xr2:uid="{B8ECCEAD-E6B2-46C2-B297-8A99F3AE59DD}"/>
   </bookViews>
   <sheets>
     <sheet name="CartData" sheetId="1" r:id="rId1"/>
@@ -558,7 +558,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>11</v>
@@ -578,7 +578,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>11</v>

</xml_diff>